<commit_message>
update feedback excel file + minor formatting fix
</commit_message>
<xml_diff>
--- a/site/Feedback_Kommentierungsvorlage_MIO-Laborbefund_100-update.xlsx
+++ b/site/Feedback_Kommentierungsvorlage_MIO-Laborbefund_100-update.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\MIO-Programm\04_MIO_Projekte\MIO_Laborbefund\01_MIO_Laborbefund_V1.0.0\06_Zwischenveröffentlichungen\02_Update_Sommer_2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CEDCD7B-6537-4B3F-90D7-30AC6B7C20F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{676C8C99-3EA6-4C5F-BEA8-AE6BD91E3324}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="22920" windowHeight="13755" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Kommentare" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="146">
   <si>
     <t>Version:</t>
   </si>
@@ -62,33 +62,18 @@
 </t>
   </si>
   <si>
-    <t>Priorität</t>
-  </si>
-  <si>
     <t>Änderungsvorschlag</t>
   </si>
   <si>
     <t>FHIR-Artefakt</t>
   </si>
   <si>
-    <t>hoch</t>
-  </si>
-  <si>
-    <t>mittel</t>
-  </si>
-  <si>
-    <t>gering</t>
-  </si>
-  <si>
     <t>Frage</t>
   </si>
   <si>
     <t>Technische Korrektur</t>
   </si>
   <si>
-    <t>Veröffentlichung des Kommentars / Änderungsvorschlags</t>
-  </si>
-  <si>
     <t>KBV_PR_MIO_LAB_BodyStructure</t>
   </si>
   <si>
@@ -240,18 +225,6 @@
   </si>
   <si>
     <t>Umsetzungsanforderungen</t>
-  </si>
-  <si>
-    <t>Unterstützungsleistungen zur LOINC-Einführung</t>
-  </si>
-  <si>
-    <t>Validierungspaket</t>
-  </si>
-  <si>
-    <t>Ja</t>
-  </si>
-  <si>
-    <t>Nein</t>
   </si>
   <si>
     <t>KBV_CS_MIO_LAB_Laboratory_Identificator</t>
@@ -750,7 +723,7 @@
     <cellStyle name="Link" xfId="1" builtinId="8"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="19">
+  <dxfs count="18">
     <dxf>
       <font>
         <b/>
@@ -830,24 +803,6 @@
     </dxf>
     <dxf>
       <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
         <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
@@ -1281,33 +1236,23 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{FFF4E8EC-4F30-47A8-A3A2-AAC268BE2CEF}" name="Tabelle9" displayName="Tabelle9" ref="A6:H107" totalsRowShown="0" headerRowDxfId="18" dataDxfId="16" headerRowBorderDxfId="17" tableBorderDxfId="15" totalsRowBorderDxfId="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{FFF4E8EC-4F30-47A8-A3A2-AAC268BE2CEF}" name="Tabelle9" displayName="Tabelle9" ref="A6:H107" totalsRowShown="0" headerRowDxfId="17" dataDxfId="15" headerRowBorderDxfId="16" tableBorderDxfId="14" totalsRowBorderDxfId="13">
   <autoFilter ref="A6:H107" xr:uid="{FFF4E8EC-4F30-47A8-A3A2-AAC268BE2CEF}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{9F9E7958-0726-40A8-852E-88BC36587309}" name="Organisation" dataDxfId="13"/>
-    <tableColumn id="2" xr3:uid="{C41BE015-F4A3-4EC1-89DD-47B946DAE8E4}" name="Kommentartyp_x000a_" dataDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{84954DFD-FC54-437E-889B-44A74D0C47C5}" name="IG-Seite" dataDxfId="11"/>
-    <tableColumn id="5" xr3:uid="{D3F757A4-6F73-44D9-8FF5-0415056993C0}" name="Informationsmodell-Struktur" dataDxfId="10"/>
-    <tableColumn id="6" xr3:uid="{2867CC53-3AC2-4C93-B15A-948E53842DD6}" name="FHIR®-Profil / Erweiterung" dataDxfId="9"/>
-    <tableColumn id="7" xr3:uid="{5C7F4A16-D9FA-4AB0-A3F2-2B6C30076F05}" name="Terminologie" dataDxfId="8"/>
-    <tableColumn id="8" xr3:uid="{EF647976-5796-4C5F-902B-6C5F5F0E591E}" name="Kommentar" dataDxfId="7"/>
-    <tableColumn id="9" xr3:uid="{C1DC4319-C81B-4B90-B152-4A25BA62E7C8}" name="Änderungsvorschlag" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{9F9E7958-0726-40A8-852E-88BC36587309}" name="Organisation" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{C41BE015-F4A3-4EC1-89DD-47B946DAE8E4}" name="Kommentartyp_x000a_" dataDxfId="11"/>
+    <tableColumn id="4" xr3:uid="{84954DFD-FC54-437E-889B-44A74D0C47C5}" name="IG-Seite" dataDxfId="10"/>
+    <tableColumn id="5" xr3:uid="{D3F757A4-6F73-44D9-8FF5-0415056993C0}" name="Informationsmodell-Struktur" dataDxfId="9"/>
+    <tableColumn id="6" xr3:uid="{2867CC53-3AC2-4C93-B15A-948E53842DD6}" name="FHIR®-Profil / Erweiterung" dataDxfId="8"/>
+    <tableColumn id="7" xr3:uid="{5C7F4A16-D9FA-4AB0-A3F2-2B6C30076F05}" name="Terminologie" dataDxfId="7"/>
+    <tableColumn id="8" xr3:uid="{EF647976-5796-4C5F-902B-6C5F5F0E591E}" name="Kommentar" dataDxfId="6"/>
+    <tableColumn id="9" xr3:uid="{C1DC4319-C81B-4B90-B152-4A25BA62E7C8}" name="Änderungsvorschlag" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D62E52BD-39E2-4189-89A4-56659D306EA2}" name="Tabelle1" displayName="Tabelle1" ref="C2:C5" totalsRowShown="0" headerRowDxfId="5">
-  <autoFilter ref="C2:C5" xr:uid="{D62E52BD-39E2-4189-89A4-56659D306EA2}"/>
-  <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{F984023E-0E5A-41D6-9BD4-C093F326259D}" name="Priorität"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4ABBED64-A846-4DB3-8FE7-156C5B67D5A0}" name="Tabelle4" displayName="Tabelle4" ref="A2:A6" totalsRowShown="0" headerRowDxfId="4">
   <autoFilter ref="A2:A6" xr:uid="{4ABBED64-A846-4DB3-8FE7-156C5B67D5A0}"/>
   <tableColumns count="1">
@@ -1317,9 +1262,9 @@
 </table>
 </file>
 
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{7DCA92C7-AF31-41FC-A1A0-C64566341CDC}" name="Tabelle5" displayName="Tabelle5" ref="I2:I40" totalsRowShown="0">
-  <autoFilter ref="I2:I40" xr:uid="{7DCA92C7-AF31-41FC-A1A0-C64566341CDC}"/>
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{7DCA92C7-AF31-41FC-A1A0-C64566341CDC}" name="Tabelle5" displayName="Tabelle5" ref="G2:G40" totalsRowShown="0">
+  <autoFilter ref="G2:G40" xr:uid="{7DCA92C7-AF31-41FC-A1A0-C64566341CDC}"/>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{8DE0297F-B3CB-43BF-807E-0BF1E0CA6389}" name="FHIR-Artefakt"/>
   </tableColumns>
@@ -1327,11 +1272,11 @@
 </table>
 </file>
 
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{C9BC38CE-2B22-4854-A781-FABC72A09216}" name="Tabelle6" displayName="Tabelle6" ref="E2:E20" totalsRowShown="0" headerRowDxfId="3">
-  <autoFilter ref="E2:E20" xr:uid="{C9BC38CE-2B22-4854-A781-FABC72A09216}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="E3:E20">
-    <sortCondition ref="E3:E20"/>
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{C9BC38CE-2B22-4854-A781-FABC72A09216}" name="Tabelle6" displayName="Tabelle6" ref="C2:C18" totalsRowShown="0" headerRowDxfId="3">
+  <autoFilter ref="C2:C18" xr:uid="{C9BC38CE-2B22-4854-A781-FABC72A09216}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C3:C18">
+    <sortCondition ref="C3:C18"/>
   </sortState>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{24A874A2-0ABE-4B1E-A80D-C0D9EB10F6E8}" name="IG-Seite"/>
@@ -1340,21 +1285,11 @@
 </table>
 </file>
 
-<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{0CB37E25-FBB9-4DFF-9BF3-C6E19FE7F2B2}" name="Tabelle7" displayName="Tabelle7" ref="M2:M4" totalsRowShown="0">
-  <autoFilter ref="M2:M4" xr:uid="{0CB37E25-FBB9-4DFF-9BF3-C6E19FE7F2B2}"/>
-  <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{CA0B2737-F7BD-4353-9A39-50C627CCC55E}" name="Veröffentlichung des Kommentars / Änderungsvorschlags"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{14B4EDD3-23A6-4C34-A6EE-8FED1C82F23E}" name="Tabelle2" displayName="Tabelle2" ref="K2:K56" totalsRowShown="0" headerRowDxfId="2">
-  <autoFilter ref="K2:K56" xr:uid="{14B4EDD3-23A6-4C34-A6EE-8FED1C82F23E}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="K3:K56">
-    <sortCondition ref="K3:K56"/>
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{14B4EDD3-23A6-4C34-A6EE-8FED1C82F23E}" name="Tabelle2" displayName="Tabelle2" ref="I2:I56" totalsRowShown="0" headerRowDxfId="2">
+  <autoFilter ref="I2:I56" xr:uid="{14B4EDD3-23A6-4C34-A6EE-8FED1C82F23E}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="I3:I56">
+    <sortCondition ref="I3:I56"/>
   </sortState>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{E9C1226E-96E7-4662-A47A-043FA8436B14}" name="Terminologie" dataDxfId="1"/>
@@ -1363,11 +1298,11 @@
 </table>
 </file>
 
-<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{826B8AE9-4B3B-40A2-A1F9-B47AD0EFEABC}" name="Tabelle3" displayName="Tabelle3" ref="G2:G22" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="G2:G22" xr:uid="{826B8AE9-4B3B-40A2-A1F9-B47AD0EFEABC}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="G3:G22">
-    <sortCondition ref="G3:G22"/>
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{826B8AE9-4B3B-40A2-A1F9-B47AD0EFEABC}" name="Tabelle3" displayName="Tabelle3" ref="E2:E22" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="E2:E22" xr:uid="{826B8AE9-4B3B-40A2-A1F9-B47AD0EFEABC}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="E3:E22">
+    <sortCondition ref="E3:E22"/>
   </sortState>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{E1299037-28C1-4C5B-9A19-E6B63CEA69AD}" name="Informationsmodell Struktur"/>
@@ -1736,22 +1671,22 @@
         <v>9</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="D6" s="22" t="s">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="E6" s="22" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="F6" s="22" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="G6" s="22" t="s">
         <v>6</v>
       </c>
       <c r="H6" s="22" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I6" s="1"/>
       <c r="J6" s="1"/>
@@ -2779,13 +2714,7 @@
   </tableParts>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="6">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000000000000}">
-          <x14:formula1>
-            <xm:f>'Drop-down menu'!$C$3:$C$4</xm:f>
-          </x14:formula1>
-          <xm:sqref>H68:H107 H7:H55</xm:sqref>
-        </x14:dataValidation>
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="5">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{4E5E5519-BD36-4565-A39D-1C6476F2FD81}">
           <x14:formula1>
             <xm:f>'Drop-down menu'!$A$3:$A$6</xm:f>
@@ -2794,25 +2723,25 @@
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{A0A2A4D4-24FE-457F-9527-38A1AF8EE766}">
           <x14:formula1>
-            <xm:f>'Drop-down menu'!$I$3:$I$40</xm:f>
+            <xm:f>'Drop-down menu'!$G$3:$G$40</xm:f>
           </x14:formula1>
           <xm:sqref>E7:E107</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{72B574A8-F4F5-45F4-ABB9-C35977BF145D}">
           <x14:formula1>
-            <xm:f>'Drop-down menu'!$G$3:$G$22</xm:f>
+            <xm:f>'Drop-down menu'!$E$3:$E$22</xm:f>
           </x14:formula1>
           <xm:sqref>D7:D107</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{6B062B74-A186-4480-946B-767C21840855}">
           <x14:formula1>
-            <xm:f>'Drop-down menu'!$K$3:$K$56</xm:f>
+            <xm:f>'Drop-down menu'!$I$3:$I$56</xm:f>
           </x14:formula1>
           <xm:sqref>F7:F107</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{7C449AFB-BB35-458C-B32D-D6D2B0433CA2}">
           <x14:formula1>
-            <xm:f>'Drop-down menu'!$E$3:$E$20</xm:f>
+            <xm:f>'Drop-down menu'!$C$3:$C$18</xm:f>
           </x14:formula1>
           <xm:sqref>C7:C107</xm:sqref>
         </x14:dataValidation>
@@ -2824,732 +2753,700 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A2:M64"/>
+  <dimension ref="A2:J64"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="52.125" customWidth="1"/>
     <col min="2" max="2" width="3.5" customWidth="1"/>
-    <col min="3" max="3" width="11" customWidth="1"/>
+    <col min="3" max="3" width="43.625" customWidth="1"/>
     <col min="4" max="4" width="2.875" customWidth="1"/>
-    <col min="5" max="5" width="43.625" customWidth="1"/>
-    <col min="6" max="6" width="2.875" customWidth="1"/>
-    <col min="7" max="7" width="52" customWidth="1"/>
-    <col min="8" max="8" width="3.75" customWidth="1"/>
+    <col min="5" max="5" width="52" customWidth="1"/>
+    <col min="6" max="6" width="3.75" customWidth="1"/>
+    <col min="7" max="7" width="70.875" customWidth="1"/>
+    <col min="8" max="8" width="6.75" customWidth="1"/>
     <col min="9" max="9" width="70.875" customWidth="1"/>
-    <col min="10" max="10" width="6.75" customWidth="1"/>
-    <col min="11" max="11" width="70.875" customWidth="1"/>
-    <col min="12" max="12" width="12.625" customWidth="1"/>
-    <col min="13" max="13" width="53.75" customWidth="1"/>
+    <col min="10" max="10" width="12.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:13" ht="15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A2" s="16" t="s">
         <v>8</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>10</v>
+        <v>69</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>80</v>
-      </c>
+        <v>71</v>
+      </c>
+      <c r="G2" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="H2" s="17"/>
       <c r="I2" s="17" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
         <v>12</v>
       </c>
-      <c r="J2" s="17"/>
-      <c r="K2" s="17" t="s">
-        <v>149</v>
-      </c>
-      <c r="M2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>16</v>
-      </c>
       <c r="C3" t="s">
-        <v>13</v>
+        <v>57</v>
       </c>
       <c r="E3" t="s">
-        <v>62</v>
+        <v>121</v>
       </c>
       <c r="G3" t="s">
-        <v>130</v>
+        <v>38</v>
       </c>
       <c r="I3" t="s">
-        <v>43</v>
-      </c>
-      <c r="K3" t="s">
-        <v>81</v>
-      </c>
-      <c r="M3" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>6</v>
       </c>
       <c r="C4" t="s">
+        <v>56</v>
+      </c>
+      <c r="E4" t="s">
+        <v>127</v>
+      </c>
+      <c r="G4" t="s">
+        <v>39</v>
+      </c>
+      <c r="I4" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" t="s">
+        <v>60</v>
+      </c>
+      <c r="E5" t="s">
+        <v>122</v>
+      </c>
+      <c r="G5" t="s">
+        <v>40</v>
+      </c>
+      <c r="I5" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" t="s">
+        <v>142</v>
+      </c>
+      <c r="E6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G6" t="s">
+        <v>41</v>
+      </c>
+      <c r="I6" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="C7" t="s">
+        <v>63</v>
+      </c>
+      <c r="E7" t="s">
+        <v>128</v>
+      </c>
+      <c r="G7" t="s">
+        <v>42</v>
+      </c>
+      <c r="I7" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="C8" t="s">
+        <v>144</v>
+      </c>
+      <c r="E8" t="s">
+        <v>124</v>
+      </c>
+      <c r="G8" t="s">
+        <v>43</v>
+      </c>
+      <c r="I8" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="C9" t="s">
+        <v>58</v>
+      </c>
+      <c r="E9" t="s">
+        <v>129</v>
+      </c>
+      <c r="G9" t="s">
+        <v>44</v>
+      </c>
+      <c r="I9" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="C10" t="s">
+        <v>61</v>
+      </c>
+      <c r="E10" t="s">
+        <v>125</v>
+      </c>
+      <c r="G10" t="s">
+        <v>45</v>
+      </c>
+      <c r="I10" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="C11" t="s">
+        <v>62</v>
+      </c>
+      <c r="E11" t="s">
+        <v>130</v>
+      </c>
+      <c r="G11" t="s">
+        <v>46</v>
+      </c>
+      <c r="I11" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="C12" t="s">
+        <v>141</v>
+      </c>
+      <c r="E12" t="s">
+        <v>131</v>
+      </c>
+      <c r="G12" t="s">
+        <v>47</v>
+      </c>
+      <c r="I12" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="C13" t="s">
+        <v>55</v>
+      </c>
+      <c r="E13" t="s">
+        <v>132</v>
+      </c>
+      <c r="G13" t="s">
+        <v>48</v>
+      </c>
+      <c r="I13" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="C14" t="s">
+        <v>143</v>
+      </c>
+      <c r="E14" t="s">
+        <v>133</v>
+      </c>
+      <c r="G14" t="s">
+        <v>49</v>
+      </c>
+      <c r="I14" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="C15" t="s">
+        <v>53</v>
+      </c>
+      <c r="E15" t="s">
+        <v>135</v>
+      </c>
+      <c r="G15" t="s">
+        <v>50</v>
+      </c>
+      <c r="I15" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="C16" t="s">
+        <v>64</v>
+      </c>
+      <c r="E16" t="s">
+        <v>134</v>
+      </c>
+      <c r="G16" t="s">
+        <v>51</v>
+      </c>
+      <c r="I16" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="C17" t="s">
+        <v>59</v>
+      </c>
+      <c r="E17" t="s">
+        <v>136</v>
+      </c>
+      <c r="G17" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="E4" t="s">
-        <v>61</v>
-      </c>
-      <c r="G4" t="s">
-        <v>136</v>
-      </c>
-      <c r="I4" t="s">
-        <v>44</v>
-      </c>
-      <c r="K4" t="s">
-        <v>114</v>
-      </c>
-      <c r="M4" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="I17" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="C18" t="s">
+        <v>54</v>
+      </c>
+      <c r="E18" t="s">
+        <v>3</v>
+      </c>
+      <c r="G18" t="s">
         <v>15</v>
       </c>
-      <c r="E5" t="s">
+      <c r="I18" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E19" t="s">
+        <v>126</v>
+      </c>
+      <c r="F19" s="3"/>
+      <c r="G19" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="I19" t="s">
         <v>65</v>
       </c>
-      <c r="G5" t="s">
-        <v>131</v>
-      </c>
-      <c r="I5" t="s">
-        <v>45</v>
-      </c>
-      <c r="K5" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E20" t="s">
+        <v>137</v>
+      </c>
+      <c r="F20" s="3"/>
+      <c r="G20" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="E6" t="s">
-        <v>151</v>
-      </c>
-      <c r="G6" t="s">
-        <v>132</v>
-      </c>
-      <c r="I6" t="s">
-        <v>46</v>
-      </c>
-      <c r="K6" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="E7" t="s">
+      <c r="I20" t="s">
         <v>68</v>
       </c>
-      <c r="G7" t="s">
-        <v>137</v>
-      </c>
-      <c r="I7" t="s">
-        <v>47</v>
-      </c>
-      <c r="K7" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="E8" t="s">
-        <v>153</v>
-      </c>
-      <c r="G8" t="s">
-        <v>133</v>
-      </c>
-      <c r="I8" t="s">
-        <v>48</v>
-      </c>
-      <c r="K8" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="E9" t="s">
-        <v>63</v>
-      </c>
-      <c r="G9" t="s">
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E21" t="s">
         <v>138</v>
       </c>
-      <c r="I9" t="s">
-        <v>49</v>
-      </c>
-      <c r="K9" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="E10" t="s">
+      <c r="F21" s="3"/>
+      <c r="G21" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="I21" t="s">
         <v>66</v>
       </c>
-      <c r="G10" t="s">
-        <v>134</v>
-      </c>
-      <c r="I10" t="s">
-        <v>50</v>
-      </c>
-      <c r="K10" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="E11" t="s">
-        <v>67</v>
-      </c>
-      <c r="G11" t="s">
-        <v>139</v>
-      </c>
-      <c r="I11" t="s">
-        <v>51</v>
-      </c>
-      <c r="K11" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="E12" t="s">
-        <v>150</v>
-      </c>
-      <c r="G12" t="s">
-        <v>140</v>
-      </c>
-      <c r="I12" t="s">
-        <v>52</v>
-      </c>
-      <c r="K12" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="E13" t="s">
-        <v>60</v>
-      </c>
-      <c r="G13" t="s">
-        <v>141</v>
-      </c>
-      <c r="I13" t="s">
-        <v>53</v>
-      </c>
-      <c r="K13" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="E14" t="s">
-        <v>152</v>
-      </c>
-      <c r="G14" t="s">
-        <v>142</v>
-      </c>
-      <c r="I14" t="s">
-        <v>54</v>
-      </c>
-      <c r="K14" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="E15" t="s">
-        <v>58</v>
-      </c>
-      <c r="G15" t="s">
-        <v>144</v>
-      </c>
-      <c r="I15" t="s">
-        <v>55</v>
-      </c>
-      <c r="K15" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="E16" t="s">
-        <v>69</v>
-      </c>
-      <c r="G16" t="s">
-        <v>143</v>
-      </c>
-      <c r="I16" t="s">
-        <v>56</v>
-      </c>
-      <c r="K16" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="E17" t="s">
-        <v>70</v>
-      </c>
-      <c r="G17" t="s">
-        <v>145</v>
-      </c>
-      <c r="I17" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="K17" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="E18" t="s">
-        <v>64</v>
-      </c>
-      <c r="G18" t="s">
-        <v>3</v>
-      </c>
-      <c r="I18" t="s">
-        <v>20</v>
-      </c>
-      <c r="K18" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="E19" t="s">
-        <v>71</v>
-      </c>
-      <c r="G19" t="s">
-        <v>135</v>
-      </c>
-      <c r="H19" s="3"/>
-      <c r="I19" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="K19" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="E20" t="s">
-        <v>59</v>
-      </c>
-      <c r="G20" t="s">
-        <v>146</v>
-      </c>
-      <c r="H20" s="3"/>
-      <c r="I20" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="K20" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="G21" t="s">
-        <v>147</v>
-      </c>
-      <c r="H21" s="3"/>
-      <c r="I21" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="K21" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A22" s="6"/>
       <c r="B22" t="s">
         <v>1</v>
       </c>
-      <c r="G22" t="s">
-        <v>148</v>
-      </c>
-      <c r="H22" s="3"/>
-      <c r="I22" s="5" t="s">
+      <c r="E22" t="s">
+        <v>139</v>
+      </c>
+      <c r="F22" s="3"/>
+      <c r="G22" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="I22" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A23" s="3"/>
+      <c r="C23" s="3"/>
+      <c r="F23" s="3"/>
+      <c r="G23" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I23" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A24" s="3"/>
+      <c r="C24" s="3"/>
+      <c r="G24" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="I24" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A25" s="3"/>
+      <c r="C25" s="3"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="I25" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A26" s="3"/>
+      <c r="C26" s="3"/>
+      <c r="F26" s="3"/>
+      <c r="G26" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="I26" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A27" s="3"/>
+      <c r="C27" s="3"/>
+      <c r="F27" s="3"/>
+      <c r="G27" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="K22" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A23" s="3"/>
-      <c r="H23" s="3"/>
-      <c r="I23" s="5" t="s">
+      <c r="I27" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="F28" s="3"/>
+      <c r="G28" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="K23" t="s">
+      <c r="I28" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A29" s="3"/>
+      <c r="C29" s="3"/>
+      <c r="F29" s="3"/>
+      <c r="G29" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="I29" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A30" s="3"/>
+      <c r="C30" s="3"/>
+      <c r="F30" s="3"/>
+      <c r="G30" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="I30" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A31" s="3"/>
+      <c r="C31" s="3"/>
+      <c r="G31" s="18" t="s">
+        <v>27</v>
+      </c>
+      <c r="I31" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A32" s="3"/>
+      <c r="C32" s="3"/>
+      <c r="F32" s="3"/>
+      <c r="G32" t="s">
+        <v>29</v>
+      </c>
+      <c r="I32" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A24" s="3"/>
-      <c r="I24" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="K24" t="s">
+      <c r="J32" s="4"/>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A33" s="3"/>
+      <c r="C33" s="3"/>
+      <c r="F33" s="5"/>
+      <c r="G33" t="s">
+        <v>30</v>
+      </c>
+      <c r="I33" t="s">
+        <v>102</v>
+      </c>
+      <c r="J33" s="4"/>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A34" s="3"/>
+      <c r="C34" s="3"/>
+      <c r="F34" s="5"/>
+      <c r="G34" t="s">
+        <v>31</v>
+      </c>
+      <c r="I34" t="s">
+        <v>79</v>
+      </c>
+      <c r="J34" s="4"/>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A35" s="3"/>
+      <c r="C35" s="3"/>
+      <c r="F35" s="5"/>
+      <c r="G35" t="s">
+        <v>32</v>
+      </c>
+      <c r="I35" t="s">
+        <v>89</v>
+      </c>
+      <c r="J35" s="4"/>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="F36" s="5"/>
+      <c r="G36" t="s">
+        <v>33</v>
+      </c>
+      <c r="I36" t="s">
+        <v>90</v>
+      </c>
+      <c r="J36" s="4"/>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A37" s="3"/>
+      <c r="C37" s="3"/>
+      <c r="F37" s="5"/>
+      <c r="G37" t="s">
+        <v>34</v>
+      </c>
+      <c r="I37" t="s">
+        <v>92</v>
+      </c>
+      <c r="J37" s="4"/>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A38" s="5"/>
+      <c r="C38" s="5"/>
+      <c r="F38" s="5"/>
+      <c r="G38" t="s">
+        <v>35</v>
+      </c>
+      <c r="I38" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="J38" s="4"/>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A39" s="5"/>
+      <c r="C39" s="5"/>
+      <c r="F39" s="5"/>
+      <c r="G39" t="s">
+        <v>36</v>
+      </c>
+      <c r="I39" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="J39" s="4"/>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A40" s="5"/>
+      <c r="C40" s="5"/>
+      <c r="F40" s="5"/>
+      <c r="G40" t="s">
+        <v>37</v>
+      </c>
+      <c r="I40" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A41" s="5"/>
+      <c r="C41" s="5"/>
+      <c r="F41" s="5"/>
+      <c r="I41" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A42" s="5"/>
+      <c r="C42" s="5"/>
+      <c r="F42" s="3"/>
+      <c r="I42" s="5" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A43" s="5"/>
+      <c r="C43" s="5"/>
+      <c r="F43" s="5"/>
+      <c r="I43" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A44" s="5"/>
+      <c r="C44" s="5"/>
+      <c r="F44" s="5"/>
+      <c r="I44" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A45" s="5"/>
+      <c r="C45" s="5"/>
+      <c r="F45" s="5"/>
+      <c r="I45" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="C46" s="5"/>
+      <c r="F46" s="5"/>
+      <c r="I46" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="C47" s="5"/>
+      <c r="F47" s="3"/>
+      <c r="I47" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="C48" s="5"/>
+      <c r="F48" s="5"/>
+      <c r="I48" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="49" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C49" s="5"/>
+      <c r="F49" s="5"/>
+      <c r="I49" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="50" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C50" s="5"/>
+      <c r="F50" s="5"/>
+      <c r="H50" s="5"/>
+      <c r="I50" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A25" s="3"/>
-      <c r="E25" s="3"/>
-      <c r="H25" s="3"/>
-      <c r="I25" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="K25" t="s">
+    <row r="51" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C51" s="5"/>
+      <c r="F51" s="3"/>
+      <c r="I51" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A26" s="3"/>
-      <c r="E26" s="3"/>
-      <c r="H26" s="3"/>
-      <c r="I26" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="K26" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A27" s="3"/>
-      <c r="E27" s="3"/>
-      <c r="H27" s="3"/>
-      <c r="I27" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="K27" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="E28" s="3"/>
-      <c r="H28" s="3"/>
-      <c r="I28" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="K28" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A29" s="3"/>
-      <c r="E29" s="3"/>
-      <c r="H29" s="3"/>
-      <c r="I29" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="K29" t="s">
+    <row r="52" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C52" s="5"/>
+      <c r="F52" s="5"/>
+      <c r="H52" s="5"/>
+      <c r="I52" s="5" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A30" s="3"/>
-      <c r="H30" s="3"/>
-      <c r="I30" s="18" t="s">
-        <v>33</v>
-      </c>
-      <c r="K30" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A31" s="3"/>
-      <c r="E31" s="3"/>
-      <c r="I31" s="18" t="s">
-        <v>32</v>
-      </c>
-      <c r="K31" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A32" s="3"/>
-      <c r="E32" s="3"/>
-      <c r="H32" s="3"/>
-      <c r="I32" t="s">
-        <v>34</v>
-      </c>
-      <c r="K32" t="s">
-        <v>122</v>
-      </c>
-      <c r="L32" s="4"/>
-    </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A33" s="3"/>
-      <c r="E33" s="3"/>
-      <c r="H33" s="5"/>
-      <c r="I33" t="s">
-        <v>35</v>
-      </c>
-      <c r="K33" t="s">
-        <v>111</v>
-      </c>
-      <c r="L33" s="4"/>
-    </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A34" s="3"/>
-      <c r="E34" s="3"/>
-      <c r="H34" s="5"/>
-      <c r="I34" t="s">
-        <v>36</v>
-      </c>
-      <c r="K34" t="s">
-        <v>88</v>
-      </c>
-      <c r="L34" s="4"/>
-    </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A35" s="3"/>
-      <c r="E35" s="3"/>
-      <c r="H35" s="5"/>
-      <c r="I35" t="s">
-        <v>37</v>
-      </c>
-      <c r="K35" t="s">
+    <row r="53" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C53" s="5"/>
+      <c r="F53" s="5"/>
+      <c r="H53" s="5"/>
+      <c r="I53" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="54" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C54" s="5"/>
+      <c r="F54" s="3"/>
+      <c r="H54" s="5"/>
+      <c r="I54" s="5" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="55" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C55" s="3"/>
+      <c r="F55" s="5"/>
+      <c r="H55" s="5"/>
+      <c r="I55" s="5" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="56" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C56" s="5"/>
+      <c r="F56" s="5"/>
+      <c r="H56" s="5"/>
+      <c r="I56" t="s">
         <v>98</v>
       </c>
-      <c r="L35" s="4"/>
-    </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="E36" s="3"/>
-      <c r="H36" s="5"/>
-      <c r="I36" t="s">
-        <v>38</v>
-      </c>
-      <c r="K36" t="s">
-        <v>99</v>
-      </c>
-      <c r="L36" s="4"/>
-    </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A37" s="3"/>
-      <c r="E37" s="3"/>
-      <c r="H37" s="5"/>
-      <c r="I37" t="s">
-        <v>39</v>
-      </c>
-      <c r="K37" t="s">
-        <v>101</v>
-      </c>
-      <c r="L37" s="4"/>
-    </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A38" s="5"/>
-      <c r="H38" s="5"/>
-      <c r="I38" t="s">
-        <v>40</v>
-      </c>
-      <c r="K38" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="L38" s="4"/>
-    </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A39" s="5"/>
-      <c r="E39" s="3"/>
-      <c r="H39" s="5"/>
-      <c r="I39" t="s">
-        <v>41</v>
-      </c>
-      <c r="K39" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="L39" s="4"/>
-    </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A40" s="5"/>
-      <c r="E40" s="5"/>
-      <c r="H40" s="5"/>
-      <c r="I40" t="s">
-        <v>42</v>
-      </c>
-      <c r="K40" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A41" s="5"/>
-      <c r="E41" s="5"/>
-      <c r="H41" s="5"/>
-      <c r="K41" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A42" s="5"/>
-      <c r="E42" s="5"/>
-      <c r="H42" s="3"/>
-      <c r="K42" s="5" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A43" s="5"/>
-      <c r="E43" s="5"/>
-      <c r="H43" s="5"/>
-      <c r="K43" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A44" s="5"/>
-      <c r="E44" s="5"/>
-      <c r="H44" s="5"/>
-      <c r="K44" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A45" s="5"/>
-      <c r="E45" s="5"/>
-      <c r="H45" s="5"/>
-      <c r="K45" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="E46" s="5"/>
-      <c r="H46" s="5"/>
-      <c r="K46" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="E47" s="5"/>
-      <c r="H47" s="3"/>
-      <c r="K47" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="E48" s="5"/>
-      <c r="H48" s="5"/>
-      <c r="K48" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="49" spans="5:12" x14ac:dyDescent="0.2">
-      <c r="E49" s="5"/>
-      <c r="H49" s="5"/>
-      <c r="K49" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="50" spans="5:12" x14ac:dyDescent="0.2">
-      <c r="E50" s="5"/>
-      <c r="H50" s="5"/>
-      <c r="J50" s="5"/>
-      <c r="K50" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="51" spans="5:12" x14ac:dyDescent="0.2">
-      <c r="E51" s="5"/>
-      <c r="H51" s="3"/>
-      <c r="K51" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="52" spans="5:12" x14ac:dyDescent="0.2">
-      <c r="E52" s="5"/>
-      <c r="H52" s="5"/>
-      <c r="J52" s="5"/>
-      <c r="K52" s="5" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="53" spans="5:12" x14ac:dyDescent="0.2">
-      <c r="E53" s="5"/>
-      <c r="H53" s="5"/>
-      <c r="J53" s="5"/>
-      <c r="K53" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="54" spans="5:12" x14ac:dyDescent="0.2">
-      <c r="E54" s="5"/>
-      <c r="H54" s="3"/>
-      <c r="J54" s="5"/>
-      <c r="K54" s="5" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="55" spans="5:12" x14ac:dyDescent="0.2">
-      <c r="E55" s="5"/>
-      <c r="H55" s="5"/>
-      <c r="J55" s="5"/>
-      <c r="K55" s="5" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="56" spans="5:12" x14ac:dyDescent="0.2">
-      <c r="E56" s="5"/>
-      <c r="H56" s="5"/>
-      <c r="J56" s="5"/>
-      <c r="K56" t="s">
-        <v>107</v>
-      </c>
-      <c r="L56" s="4"/>
-    </row>
-    <row r="57" spans="5:12" x14ac:dyDescent="0.2">
-      <c r="E57" s="3"/>
+      <c r="J56" s="4"/>
+    </row>
+    <row r="57" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C57" s="5"/>
+      <c r="F57" s="5"/>
       <c r="H57" s="5"/>
-      <c r="J57" s="5"/>
-      <c r="K57" s="5"/>
-      <c r="L57" s="4"/>
-    </row>
-    <row r="58" spans="5:12" x14ac:dyDescent="0.2">
-      <c r="E58" s="5"/>
-      <c r="J58" s="5"/>
-      <c r="K58" s="5"/>
-      <c r="L58" s="4"/>
-    </row>
-    <row r="59" spans="5:12" x14ac:dyDescent="0.2">
-      <c r="E59" s="5"/>
-      <c r="J59" s="3"/>
-      <c r="K59" s="3"/>
-    </row>
-    <row r="60" spans="5:12" x14ac:dyDescent="0.2">
-      <c r="E60" s="5"/>
-      <c r="J60" s="5"/>
-      <c r="K60" s="5"/>
-    </row>
-    <row r="61" spans="5:12" x14ac:dyDescent="0.2">
-      <c r="J61" s="5"/>
-      <c r="K61" s="5"/>
-    </row>
-    <row r="62" spans="5:12" x14ac:dyDescent="0.2">
-      <c r="J62" s="5"/>
-      <c r="K62" s="5"/>
-    </row>
-    <row r="63" spans="5:12" x14ac:dyDescent="0.2">
-      <c r="J63" s="18"/>
-      <c r="K63" s="18"/>
-    </row>
-    <row r="64" spans="5:12" x14ac:dyDescent="0.2">
-      <c r="J64" s="18"/>
-      <c r="K64" s="18"/>
+      <c r="I57" s="5"/>
+      <c r="J57" s="4"/>
+    </row>
+    <row r="58" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="C58" s="5"/>
+      <c r="H58" s="5"/>
+      <c r="I58" s="5"/>
+      <c r="J58" s="4"/>
+    </row>
+    <row r="59" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="H59" s="3"/>
+      <c r="I59" s="3"/>
+    </row>
+    <row r="60" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="H60" s="5"/>
+      <c r="I60" s="5"/>
+    </row>
+    <row r="61" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="H61" s="5"/>
+      <c r="I61" s="5"/>
+    </row>
+    <row r="62" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="H62" s="5"/>
+      <c r="I62" s="5"/>
+    </row>
+    <row r="63" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="H63" s="18"/>
+      <c r="I63" s="18"/>
+    </row>
+    <row r="64" spans="3:10" x14ac:dyDescent="0.2">
+      <c r="H64" s="18"/>
+      <c r="I64" s="18"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="I3:I7">
-    <sortCondition ref="I3:I7"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="G3:G7">
+    <sortCondition ref="G3:G7"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-  <tableParts count="7">
+  <tableParts count="5">
     <tablePart r:id="rId2"/>
     <tablePart r:id="rId3"/>
     <tablePart r:id="rId4"/>
     <tablePart r:id="rId5"/>
     <tablePart r:id="rId6"/>
-    <tablePart r:id="rId7"/>
-    <tablePart r:id="rId8"/>
   </tableParts>
 </worksheet>
 </file>
@@ -3790,6 +3687,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="9a474d83-48f9-40d7-948b-4e2374dd405a">
@@ -3798,15 +3704,6 @@
     <TaxCatchAll xmlns="86f14935-6ae9-412a-be15-d43e59e5fff2" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3829,6 +3726,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B304C4F3-8F41-455D-BC70-1AAF447B86D5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9755F0A4-AD65-4100-9027-7AF7F8B3F062}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
@@ -3843,12 +3748,4 @@
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B304C4F3-8F41-455D-BC70-1AAF447B86D5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>